<commit_message>
Add 6 questions on visual properties (色のユニバーサルデザイン)
</commit_message>
<xml_diff>
--- a/my-weakness.xlsx
+++ b/my-weakness.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="102">
   <si>
     <t>カテゴリ</t>
   </si>
@@ -284,6 +284,42 @@
   </si>
   <si>
     <t>バンク・ミケルセン ／ ノーマライゼーション</t>
+  </si>
+  <si>
+    <t>対象物に注意を向けていないときに、思わず人の目を引きつけて発見されやすい度合いのことを何というか。無彩色より有彩色、寒色系より高彩度の暖色系で高くなるが、1型色覚の人には赤が暗く見えるため配慮が必要となる。</t>
+  </si>
+  <si>
+    <t>誘目性</t>
+  </si>
+  <si>
+    <t>対象物を注視した（注意を向けて探した）ときに、その対象物の存在を確認しやすい度合いのことを何というか。背景色と対象物の色の「明度差」を大きくするほど高くなる。</t>
+  </si>
+  <si>
+    <t>視認性</t>
+  </si>
+  <si>
+    <t>複数の対象物があるときに、色や形状などの特性によってそれぞれを他と区別しやすい度合いのことを何というか。色の違いを色名で言い表せる組み合わせが有効であり、色覚特性や加齢への配慮として形や模様・文字を添える工夫が求められる。</t>
+  </si>
+  <si>
+    <t>識別性</t>
+  </si>
+  <si>
+    <t>案内表示や印刷物などの「文字や数字」の読みやすさの度合いのことを何というか。背景との明度差を大きくするほか、文字を太くしたり、セパレーションカラー（境界線・アウトライン）を入れたりすることで高められる。</t>
+  </si>
+  <si>
+    <t>可読性</t>
+  </si>
+  <si>
+    <t>ピクトグラムやサインなどの「図形」を見たときに、その形や意味を正しく理解しやすい度合いのことを何というか。視認性の一種であり、背景との明度差を大きくしたりシンプルな形状にしたりすることで高められる。</t>
+  </si>
+  <si>
+    <t>明視性</t>
+  </si>
+  <si>
+    <t>赤が「危険・お湯」、黄が「注意」、青が「安全・水」を表すように、色が持つ共通の感情効果（心理効果）を利用して、特定の状態や約束事を伝える働きを何というか。色覚特性のある人は色だけでは判別しにくい場合があるため、文字や形を併用することが重要となる。</t>
+  </si>
+  <si>
+    <t>意味性・記号性</t>
   </si>
 </sst>
 </file>
@@ -464,7 +500,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.8515625" customWidth="1"/>
@@ -978,6 +1014,72 @@
         <v>89</v>
       </c>
     </row>
+    <row r="47" ht="71.25">
+      <c r="A47" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="48" ht="57.75">
+      <c r="A48" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="49" ht="71.25">
+      <c r="A49" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="50" ht="71.25">
+      <c r="A50" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="51" ht="71.25">
+      <c r="A51" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="52" ht="84.75">
+      <c r="A52" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.699999988079071" right="0.699999988079071" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
Add question on X-linked color vision gene rates
</commit_message>
<xml_diff>
--- a/my-weakness.xlsx
+++ b/my-weakness.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="110">
   <si>
     <t>カテゴリ</t>
   </si>
@@ -338,6 +338,12 @@
   </si>
   <si>
     <t>常染色体 ／ 性染色体</t>
+  </si>
+  <si>
+    <t>日本人の場合、X染色体に色覚異常の遺伝子を持つ確率は男性と女性でそれぞれ何％か。</t>
+  </si>
+  <si>
+    <t>男性 5％ ／ 女性 10％（5％+5％）＝保因者</t>
   </si>
 </sst>
 </file>
@@ -518,7 +524,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.8515625" customWidth="1"/>
@@ -1131,6 +1137,17 @@
         <v>107</v>
       </c>
     </row>
+    <row r="56" ht="30.75">
+      <c r="A56" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.699999988079071" right="0.699999988079071" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
Add another 色誤認 question
</commit_message>
<xml_diff>
--- a/my-weakness.xlsx
+++ b/my-weakness.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="111">
   <si>
     <t>カテゴリ</t>
   </si>
@@ -344,6 +344,9 @@
   </si>
   <si>
     <t>男性 5％ ／ 女性 10％（5％+5％）＝保因者</t>
+  </si>
+  <si>
+    <t>1型・2型色覚の人が「水色とピンク」「深緑と焦茶」「緑とグレー」を取り違えたり、高齢者が水晶体の黄変によって「白と黄色」「黒と紺」を取り違えたりするように、本来の色とは異なる色として認識してしまうことを何というか。</t>
   </si>
 </sst>
 </file>
@@ -524,7 +527,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.8515625" customWidth="1"/>
@@ -1148,6 +1151,17 @@
         <v>109</v>
       </c>
     </row>
+    <row r="57" ht="71.25">
+      <c r="A57" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.699999988079071" right="0.699999988079071" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
Add question on hue-tone system
</commit_message>
<xml_diff>
--- a/my-weakness.xlsx
+++ b/my-weakness.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="113">
   <si>
     <t>カテゴリ</t>
   </si>
@@ -347,6 +347,12 @@
   </si>
   <si>
     <t>1型・2型色覚の人が「水色とピンク」「深緑と焦茶」「緑とグレー」を取り違えたり、高齢者が水晶体の黄変によって「白と黄色」「黒と紺」を取り違えたりするように、本来の色とは異なる色として認識してしまうことを何というか。</t>
+  </si>
+  <si>
+    <t>PCCSなどの「ヒュー・トーンシステム」とは、【 　】（ヒュー）と、色の持つ印象やイメージが共通する【 　】と【 　 】を1つに統合した【 　】（色調）の2つの軸で色を表す仕組みである。</t>
+  </si>
+  <si>
+    <t>色相 ／ 明度と彩度（順不同） ／ トーン</t>
   </si>
 </sst>
 </file>
@@ -527,7 +533,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.8515625" customWidth="1"/>
@@ -1162,6 +1168,17 @@
         <v>104</v>
       </c>
     </row>
+    <row r="58" ht="57.75">
+      <c r="A58" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.699999988079071" right="0.699999988079071" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
Add question on 混同色線
</commit_message>
<xml_diff>
--- a/my-weakness.xlsx
+++ b/my-weakness.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="115">
   <si>
     <t>カテゴリ</t>
   </si>
@@ -353,6 +353,12 @@
   </si>
   <si>
     <t>色相 ／ 明度と彩度（順不同） ／ トーン</t>
+  </si>
+  <si>
+    <t>色度図（馬蹄形の色の地図）上に形成される、1型色覚や2型色覚などの色覚特性のタイプごとに「区別しにくい（同じ色や似た色に見える）色の組み合わせ」を結んだ直線を何というか。</t>
+  </si>
+  <si>
+    <t>混同色線</t>
   </si>
 </sst>
 </file>
@@ -533,7 +539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.8515625" customWidth="1"/>
@@ -1179,6 +1185,17 @@
         <v>112</v>
       </c>
     </row>
+    <row r="59" ht="57.75">
+      <c r="A59" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.699999988079071" right="0.699999988079071" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
Add question on number of people with color vision deficiency in Japan
</commit_message>
<xml_diff>
--- a/my-weakness.xlsx
+++ b/my-weakness.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="117">
   <si>
     <t>カテゴリ</t>
   </si>
@@ -359,6 +359,12 @@
   </si>
   <si>
     <t>混同色線</t>
+  </si>
+  <si>
+    <t>色覚異常の人は国内にどれほどいるか。</t>
+  </si>
+  <si>
+    <t>およそ300万人</t>
   </si>
 </sst>
 </file>
@@ -539,7 +545,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.8515625" customWidth="1"/>
@@ -1196,6 +1202,17 @@
         <v>114</v>
       </c>
     </row>
+    <row r="60" ht="30.75">
+      <c r="A60" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.699999988079071" right="0.699999988079071" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
Add question on achromatic color naming
</commit_message>
<xml_diff>
--- a/my-weakness.xlsx
+++ b/my-weakness.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="119">
   <si>
     <t>カテゴリ</t>
   </si>
@@ -365,6 +365,12 @@
   </si>
   <si>
     <t>およそ300万人</t>
+  </si>
+  <si>
+    <t>1型・2型色覚の人は無彩色の場合、明度が高いと（　）、明度が低いと（　）と呼ぶ傾向がある。それぞれ色名を答えなさい。</t>
+  </si>
+  <si>
+    <t>ピンク ／ 緑</t>
   </si>
 </sst>
 </file>
@@ -545,7 +551,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.8515625" customWidth="1"/>
@@ -1213,6 +1219,17 @@
         <v>116</v>
       </c>
     </row>
+    <row r="61" ht="44.25">
+      <c r="A61" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.699999988079071" right="0.699999988079071" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
Add question on protan gray naming
</commit_message>
<xml_diff>
--- a/my-weakness.xlsx
+++ b/my-weakness.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="121">
   <si>
     <t>カテゴリ</t>
   </si>
@@ -371,6 +371,12 @@
   </si>
   <si>
     <t>ピンク ／ 緑</t>
+  </si>
+  <si>
+    <t>1型色覚の人は、（　）系の様々な色を「灰色」や「グレー」と呼ぶ傾向がある。色名は？</t>
+  </si>
+  <si>
+    <t>青緑</t>
   </si>
 </sst>
 </file>
@@ -551,7 +557,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.8515625" customWidth="1"/>
@@ -1230,6 +1236,17 @@
         <v>118</v>
       </c>
     </row>
+    <row r="62" ht="30.75">
+      <c r="A62" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.699999988079071" right="0.699999988079071" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
Add question on three attributes of color
</commit_message>
<xml_diff>
--- a/my-weakness.xlsx
+++ b/my-weakness.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="123">
   <si>
     <t>カテゴリ</t>
   </si>
@@ -377,6 +377,12 @@
   </si>
   <si>
     <t>青緑</t>
+  </si>
+  <si>
+    <t>色の3属性は？</t>
+  </si>
+  <si>
+    <t>色相 ／ 明度 ／ 彩度</t>
   </si>
 </sst>
 </file>
@@ -557,7 +563,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.8515625" customWidth="1"/>
@@ -1247,6 +1253,17 @@
         <v>120</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.699999988079071" right="0.699999988079071" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
   <pageSetup orientation="portrait"/>

</xml_diff>